<commit_message>
Paquetes regenerados de Tu Patrimonio v1.3 y Your Money v3.4 sin nombres prohibidos
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01P5F6YBSbmgYFHyY7RUeBgK
</commit_message>
<xml_diff>
--- a/cursos/tu_patrimonio/moodle/herramientas/Herramientas_TPTF.xlsx
+++ b/cursos/tu_patrimonio/moodle/herramientas/Herramientas_TPTF.xlsx
@@ -11,6 +11,7 @@
     <sheet name="Deudas" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Fondo" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Meta" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Mis bienes" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1127,4 +1128,181 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F18"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="38" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="24" customWidth="1" min="5" max="5"/>
+    <col width="24" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Lo que tengo, a nombre de quién y quién lo recibe</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>No anotes números de cuenta ni contraseñas; solo dónde está cada documento.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Bien o cuenta</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>A nombre de</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Valor aproximado</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>Documento</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>Dónde está el documento</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>Beneficiario o heredero</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="9" t="n"/>
+      <c r="B5" s="9" t="n"/>
+      <c r="C5" s="5" t="n"/>
+      <c r="D5" s="9" t="n"/>
+      <c r="E5" s="9" t="n"/>
+      <c r="F5" s="9" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="9" t="n"/>
+      <c r="B6" s="9" t="n"/>
+      <c r="C6" s="5" t="n"/>
+      <c r="D6" s="9" t="n"/>
+      <c r="E6" s="9" t="n"/>
+      <c r="F6" s="9" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="9" t="n"/>
+      <c r="B7" s="9" t="n"/>
+      <c r="C7" s="5" t="n"/>
+      <c r="D7" s="9" t="n"/>
+      <c r="E7" s="9" t="n"/>
+      <c r="F7" s="9" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="9" t="n"/>
+      <c r="B8" s="9" t="n"/>
+      <c r="C8" s="5" t="n"/>
+      <c r="D8" s="9" t="n"/>
+      <c r="E8" s="9" t="n"/>
+      <c r="F8" s="9" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="9" t="n"/>
+      <c r="B9" s="9" t="n"/>
+      <c r="C9" s="5" t="n"/>
+      <c r="D9" s="9" t="n"/>
+      <c r="E9" s="9" t="n"/>
+      <c r="F9" s="9" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="9" t="n"/>
+      <c r="B10" s="9" t="n"/>
+      <c r="C10" s="5" t="n"/>
+      <c r="D10" s="9" t="n"/>
+      <c r="E10" s="9" t="n"/>
+      <c r="F10" s="9" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="9" t="n"/>
+      <c r="B11" s="9" t="n"/>
+      <c r="C11" s="5" t="n"/>
+      <c r="D11" s="9" t="n"/>
+      <c r="E11" s="9" t="n"/>
+      <c r="F11" s="9" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="9" t="n"/>
+      <c r="B12" s="9" t="n"/>
+      <c r="C12" s="5" t="n"/>
+      <c r="D12" s="9" t="n"/>
+      <c r="E12" s="9" t="n"/>
+      <c r="F12" s="9" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="9" t="n"/>
+      <c r="B13" s="9" t="n"/>
+      <c r="C13" s="5" t="n"/>
+      <c r="D13" s="9" t="n"/>
+      <c r="E13" s="9" t="n"/>
+      <c r="F13" s="9" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="9" t="n"/>
+      <c r="B14" s="9" t="n"/>
+      <c r="C14" s="5" t="n"/>
+      <c r="D14" s="9" t="n"/>
+      <c r="E14" s="9" t="n"/>
+      <c r="F14" s="9" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="9" t="n"/>
+      <c r="B15" s="9" t="n"/>
+      <c r="C15" s="5" t="n"/>
+      <c r="D15" s="9" t="n"/>
+      <c r="E15" s="9" t="n"/>
+      <c r="F15" s="9" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="9" t="n"/>
+      <c r="B16" s="9" t="n"/>
+      <c r="C16" s="5" t="n"/>
+      <c r="D16" s="9" t="n"/>
+      <c r="E16" s="9" t="n"/>
+      <c r="F16" s="9" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="7" t="inlineStr">
+        <is>
+          <t>Valor total aproximado</t>
+        </is>
+      </c>
+      <c r="C18" s="8">
+        <f>SUM(C5:C16)</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>